<commit_message>
Add per-event timezone and custom X-property support
New features:
- Timezone field: IANA timezone per event (e.g. Europe/London,
  America/New_York) applied as TZID parameter on DTSTART/DTEND
- Custom X-properties: any unmapped CSV column with an X- prefix
  header is automatically written as an ICS extension property
- 25 mapped fields total (up from 23)

Other changes:
- About dialog updated to v1.2 with new feature list
- Sample data: replaced Car MOT with US Team Call to demonstrate
  America/New_York timezone
- Excel templates regenerated with Timezone column and updated notes
- README updated with timezone, X-property docs, and field count

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CSV2ICS_Sample.xlsx
+++ b/CSV2ICS_Sample.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$W$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$X$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W16"/>
+  <dimension ref="A1:X16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -506,6 +506,7 @@
     <col width="30" customWidth="1" min="21" max="21"/>
     <col width="30" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -624,6 +625,11 @@
           <t>Duration</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Timezone</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -717,6 +723,11 @@
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>Europe/London</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -782,6 +793,7 @@
       <c r="U3" s="3" t="inlineStr"/>
       <c r="V3" s="3" t="inlineStr"/>
       <c r="W3" s="3" t="inlineStr"/>
+      <c r="X3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -843,6 +855,7 @@
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -916,6 +929,7 @@
       <c r="U5" s="3" t="inlineStr"/>
       <c r="V5" s="3" t="inlineStr"/>
       <c r="W5" s="3" t="inlineStr"/>
+      <c r="X5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -989,6 +1003,7 @@
           <t>1 hour</t>
         </is>
       </c>
+      <c r="X6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1062,6 +1077,7 @@
         </is>
       </c>
       <c r="W7" s="3" t="inlineStr"/>
+      <c r="X7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1151,6 +1167,7 @@
           <t>2 hours</t>
         </is>
       </c>
+      <c r="X8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1228,6 +1245,7 @@
       <c r="U9" s="3" t="inlineStr"/>
       <c r="V9" s="3" t="inlineStr"/>
       <c r="W9" s="3" t="inlineStr"/>
+      <c r="X9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1317,39 +1335,40 @@
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr"/>
+      <c r="X10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Car MOT</t>
+          <t>US Team Call</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr"/>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
       <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Kwik Fit, Leeds</t>
-        </is>
-      </c>
+      <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Annual MOT test</t>
+          <t>Weekly sync with New York office</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr"/>
@@ -1358,11 +1377,7 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="L11" s="3" t="inlineStr"/>
       <c r="M11" s="3" t="inlineStr">
         <is>
           <t>OPAQUE</t>
@@ -1370,26 +1385,35 @@
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>PRIVATE</t>
+          <t>PUBLIC</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>1440</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>Weekly</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr"/>
       <c r="R11" s="3" t="inlineStr"/>
       <c r="S11" s="3" t="inlineStr"/>
       <c r="T11" s="3" t="inlineStr"/>
-      <c r="U11" s="3" t="inlineStr"/>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>us-team@company.com</t>
+        </is>
+      </c>
       <c r="V11" s="3" t="inlineStr"/>
       <c r="W11" s="3" t="inlineStr"/>
+      <c r="X11" s="3" t="inlineStr">
+        <is>
+          <t>America/New_York</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1471,6 +1495,7 @@
           <t>1.5 hours</t>
         </is>
       </c>
+      <c r="X12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1540,6 +1565,7 @@
       <c r="U13" s="3" t="inlineStr"/>
       <c r="V13" s="3" t="inlineStr"/>
       <c r="W13" s="3" t="inlineStr"/>
+      <c r="X13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1597,6 +1623,7 @@
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="inlineStr"/>
       <c r="W14" s="2" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1682,6 +1709,7 @@
           <t>30 minutes</t>
         </is>
       </c>
+      <c r="X15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1751,9 +1779,10 @@
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="inlineStr"/>
       <c r="W16" s="2" t="inlineStr"/>
+      <c r="X16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W1"/>
+  <autoFilter ref="A1:X1"/>
   <dataValidations count="5">
     <dataValidation sqref="F2:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
@@ -1782,7 +1811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2319,57 +2348,79 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Timezone</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>IANA timezone for this event</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Europe/London, America/New_York, Asia/Tokyo</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Tips:</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>• Only Title and Start Date are required. All other fields are optional.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>• Select your date format on Page 1 of CSV2ICS to match your data.</t>
+          <t>• Only Title and Start Date are required. All other fields are optional.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>• Default reminders can also be set on the Export page.</t>
+          <t>• Select your date format on Page 1 of CSV2ICS to match your data.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>• Save as CSV (UTF-8) before importing. TSV (tab-delimited) is also supported.</t>
+          <t>• Default reminders can also be set on the Export page.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>• Attendee emails should be separated by semicolons.</t>
+          <t>• Save as CSV (UTF-8) before importing. TSV (tab-delimited) is also supported.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>• Duration is used instead of End Date/Time when End Date is not provided.</t>
+          <t>• Attendee emails should be separated by semicolons.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>• Duration is used instead of End Date/Time when End Date is not provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>• Recurrence Count and End Date are mutually exclusive (RFC 5545).</t>
         </is>

</xml_diff>